<commit_message>
Finished all the Manager functions, can generate and export reports including seeing the graphs
</commit_message>
<xml_diff>
--- a/Project/Output/sales_report.xlsx
+++ b/Project/Output/sales_report.xlsx
@@ -468,27 +468,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2646.0</t>
+          <t>33173.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3373.0</t>
+          <t>33179.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4047.6</t>
+          <t>39814.8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-1401.6</t>
+          <t>-6641.8</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>-34.63</t>
+          <t>-16.68</t>
         </is>
       </c>
     </row>
@@ -500,27 +500,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3042.0</t>
+          <t>30179.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3141.0</t>
+          <t>33693.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3769.2</t>
+          <t>40431.6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-727.2</t>
+          <t>-10252.6</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>-19.29</t>
+          <t>-25.36</t>
         </is>
       </c>
     </row>
@@ -532,27 +532,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2606.0</t>
+          <t>31937.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2473.0</t>
+          <t>31671.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2967.6</t>
+          <t>38005.2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>-361.6</t>
+          <t>-6068.2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-12.18</t>
+          <t>-15.97</t>
         </is>
       </c>
     </row>
@@ -564,27 +564,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3625.0</t>
+          <t>32409.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3445.0</t>
+          <t>35435.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4134.0</t>
+          <t>42522.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>-509.0</t>
+          <t>-10113.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-12.31</t>
+          <t>-23.78</t>
         </is>
       </c>
     </row>
@@ -596,27 +596,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2295.0</t>
+          <t>33587.0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2930.0</t>
+          <t>36069.0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3516.0</t>
+          <t>43282.8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-1221.0</t>
+          <t>-9695.8</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-34.73</t>
+          <t>-22.4</t>
         </is>
       </c>
     </row>
@@ -628,27 +628,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14214.0</t>
+          <t>161285.0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15362.0</t>
+          <t>170047.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>18434.4</t>
+          <t>204056.4</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-4220.4</t>
+          <t>-42771.4</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-22.89</t>
+          <t>-20.96</t>
         </is>
       </c>
     </row>

</xml_diff>